<commit_message>
Refactor classical NLP pipeline into reusable modules
</commit_message>
<xml_diff>
--- a/logs/experiments.xlsx
+++ b/logs/experiments.xlsx
@@ -407,7 +407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="9.9296875" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -742,6 +742,103 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EXP-001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Logistic Regression</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MRPC</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>3668</v>
+      </c>
+      <c r="G4" t="n">
+        <v>408</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1725</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0.7279411764705882</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.723404255319149</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.974910394265233</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.8305343511450382</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.6758634102970187</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>0.03656619996763766</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.0009960001334547997</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TF-IDF (1,2)-gram baseline</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implement SBERT baseline for MRPC
</commit_message>
<xml_diff>
--- a/logs/experiments.xlsx
+++ b/logs/experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bevan\Desktop\Paraphrase_Detection_Generation\logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D223338-A6A9-4256-9450-7DCA1653147C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C102B2-FD1E-4F74-897B-EA16F0EC7593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1747" yWindow="1747" windowWidth="16201" windowHeight="9308" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="40">
   <si>
     <t>Experiment ID</t>
   </si>
@@ -91,42 +91,30 @@
     <t>Status</t>
   </si>
   <si>
-    <t>EXP-000</t>
-  </si>
-  <si>
-    <t>Environment Setup</t>
+    <t>EXP-001</t>
+  </si>
+  <si>
+    <t>2026-08-04</t>
+  </si>
+  <si>
+    <t>Baseline</t>
+  </si>
+  <si>
+    <t>Logistic Regression</t>
+  </si>
+  <si>
+    <t>MRPC</t>
   </si>
   <si>
     <t>N/A</t>
   </si>
   <si>
-    <t>MRPC, QQP, PAWS, MSCOCO</t>
-  </si>
-  <si>
-    <t>Project initialized, datasets downloaded and verified</t>
+    <t>TF-IDF (1,2)-gram baseline</t>
   </si>
   <si>
     <t>Completed</t>
   </si>
   <si>
-    <t>EXP-001</t>
-  </si>
-  <si>
-    <t>2026-08-04</t>
-  </si>
-  <si>
-    <t>Baseline</t>
-  </si>
-  <si>
-    <t>Logistic Regression</t>
-  </si>
-  <si>
-    <t>MRPC</t>
-  </si>
-  <si>
-    <t>TF-IDF (1,2)-gram baseline</t>
-  </si>
-  <si>
     <t>EXP-002</t>
   </si>
   <si>
@@ -137,6 +125,21 @@
   </si>
   <si>
     <t>PAWS</t>
+  </si>
+  <si>
+    <t>EXP-004</t>
+  </si>
+  <si>
+    <t>2026-08-05</t>
+  </si>
+  <si>
+    <t>SBERT Baseline</t>
+  </si>
+  <si>
+    <t>SBERT + Logistic Regression</t>
+  </si>
+  <si>
+    <t>all-MiniLM-L6-v2 (384d), concatenated embeddings</t>
   </si>
 </sst>
 </file>
@@ -180,16 +183,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -548,288 +545,288 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="85.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="3">
-        <v>46234</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="D2" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="V2" s="2" t="s">
+      <c r="E2" t="s">
         <v>27</v>
       </c>
-      <c r="W2" s="2" t="s">
-        <v>28</v>
+      <c r="F2">
+        <v>3668</v>
+      </c>
+      <c r="G2">
+        <v>408</v>
+      </c>
+      <c r="H2">
+        <v>1725</v>
+      </c>
+      <c r="I2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2">
+        <v>0.7279411764705882</v>
+      </c>
+      <c r="M2">
+        <v>0.72340425531914898</v>
+      </c>
+      <c r="N2">
+        <v>0.97491039426523296</v>
+      </c>
+      <c r="O2">
+        <v>0.83053435114503815</v>
+      </c>
+      <c r="P2">
+        <v>0.67586341029701869</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>28</v>
+      </c>
+      <c r="R2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2">
+        <v>3.6566199967637658E-2</v>
+      </c>
+      <c r="U2">
+        <v>9.9600013345479965E-4</v>
+      </c>
+      <c r="V2" t="s">
+        <v>29</v>
+      </c>
+      <c r="W2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3">
+        <v>363844</v>
+      </c>
+      <c r="G3">
+        <v>40430</v>
+      </c>
+      <c r="H3">
+        <v>390964</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3">
+        <v>0.76754884986396243</v>
+      </c>
+      <c r="M3">
+        <v>0.72284948420112094</v>
+      </c>
+      <c r="N3">
+        <v>0.59785018474974805</v>
+      </c>
+      <c r="O3">
+        <v>0.65443447565818502</v>
+      </c>
+      <c r="P3">
+        <v>0.83643592458999116</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" t="s">
+        <v>28</v>
+      </c>
+      <c r="S3" t="s">
+        <v>28</v>
+      </c>
+      <c r="T3">
+        <v>3.161926100030541</v>
+      </c>
+      <c r="U3">
+        <v>8.3405999466776848E-3</v>
+      </c>
+      <c r="V3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" t="s">
+      <c r="W3" t="s">
         <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3">
-        <v>3668</v>
-      </c>
-      <c r="G3">
-        <v>408</v>
-      </c>
-      <c r="H3">
-        <v>1725</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3">
-        <v>0.7279411764705882</v>
-      </c>
-      <c r="M3">
-        <v>0.72340425531914898</v>
-      </c>
-      <c r="N3">
-        <v>0.97491039426523296</v>
-      </c>
-      <c r="O3">
-        <v>0.83053435114503815</v>
-      </c>
-      <c r="P3">
-        <v>0.67586341029701869</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>25</v>
-      </c>
-      <c r="R3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S3" t="s">
-        <v>25</v>
-      </c>
-      <c r="T3">
-        <v>3.6566199967637658E-2</v>
-      </c>
-      <c r="U3">
-        <v>9.9600013345479965E-4</v>
-      </c>
-      <c r="V3" t="s">
-        <v>34</v>
-      </c>
-      <c r="W3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4">
+        <v>49401</v>
+      </c>
+      <c r="G4">
+        <v>8000</v>
+      </c>
+      <c r="H4">
+        <v>8000</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4">
+        <v>0.55649999999999999</v>
+      </c>
+      <c r="M4">
+        <v>0.49769112365315549</v>
+      </c>
+      <c r="N4">
+        <v>0.27408872562870867</v>
+      </c>
+      <c r="O4">
+        <v>0.35349854227405247</v>
+      </c>
+      <c r="P4">
+        <v>0.54809710277366008</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>28</v>
+      </c>
+      <c r="R4" t="s">
+        <v>28</v>
+      </c>
+      <c r="S4" t="s">
+        <v>28</v>
+      </c>
+      <c r="T4">
+        <v>0.69511909992434084</v>
+      </c>
+      <c r="U4">
+        <v>9.1748000122606754E-3</v>
+      </c>
+      <c r="V4" t="s">
+        <v>29</v>
+      </c>
+      <c r="W4" t="s">
         <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4">
-        <v>363844</v>
-      </c>
-      <c r="G4">
-        <v>40430</v>
-      </c>
-      <c r="H4">
-        <v>390964</v>
-      </c>
-      <c r="I4" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L4">
-        <v>0.76754884986396243</v>
-      </c>
-      <c r="M4">
-        <v>0.72284948420112094</v>
-      </c>
-      <c r="N4">
-        <v>0.59785018474974805</v>
-      </c>
-      <c r="O4">
-        <v>0.65443447565818502</v>
-      </c>
-      <c r="P4">
-        <v>0.83643592458999116</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>25</v>
-      </c>
-      <c r="R4" t="s">
-        <v>25</v>
-      </c>
-      <c r="S4" t="s">
-        <v>25</v>
-      </c>
-      <c r="T4">
-        <v>3.161926100030541</v>
-      </c>
-      <c r="U4">
-        <v>8.3405999466776848E-3</v>
-      </c>
-      <c r="V4" t="s">
-        <v>34</v>
-      </c>
-      <c r="W4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
         <v>37</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5">
+        <v>3668</v>
+      </c>
+      <c r="G5">
+        <v>408</v>
+      </c>
+      <c r="H5">
+        <v>1725</v>
+      </c>
+      <c r="I5">
+        <v>32</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L5">
+        <v>0.62990196078431371</v>
+      </c>
+      <c r="M5">
+        <v>0.72068965517241379</v>
+      </c>
+      <c r="N5">
+        <v>0.74910394265232971</v>
+      </c>
+      <c r="O5">
+        <v>0.73462214411247806</v>
+      </c>
+      <c r="P5">
+        <v>0.56127920869106163</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T5">
+        <v>0.7937600000295788</v>
+      </c>
+      <c r="U5">
+        <v>3.4654999617487192E-3</v>
+      </c>
+      <c r="V5" t="s">
+        <v>39</v>
+      </c>
+      <c r="W5" t="s">
         <v>30</v>
-      </c>
-      <c r="C5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F5">
-        <v>49401</v>
-      </c>
-      <c r="G5">
-        <v>8000</v>
-      </c>
-      <c r="H5">
-        <v>8000</v>
-      </c>
-      <c r="I5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J5" t="s">
-        <v>25</v>
-      </c>
-      <c r="K5" t="s">
-        <v>25</v>
-      </c>
-      <c r="L5">
-        <v>0.55649999999999999</v>
-      </c>
-      <c r="M5">
-        <v>0.49769112365315549</v>
-      </c>
-      <c r="N5">
-        <v>0.27408872562870867</v>
-      </c>
-      <c r="O5">
-        <v>0.35349854227405247</v>
-      </c>
-      <c r="P5">
-        <v>0.54809710277366008</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>25</v>
-      </c>
-      <c r="R5" t="s">
-        <v>25</v>
-      </c>
-      <c r="S5" t="s">
-        <v>25</v>
-      </c>
-      <c r="T5">
-        <v>0.69511909992434084</v>
-      </c>
-      <c r="U5">
-        <v>9.1748000122606754E-3</v>
-      </c>
-      <c r="V5" t="s">
-        <v>34</v>
-      </c>
-      <c r="W5" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add DistilBERT implementation for MRPC
</commit_message>
<xml_diff>
--- a/logs/experiments.xlsx
+++ b/logs/experiments.xlsx
@@ -401,7 +401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="9.9296875" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -1100,6 +1100,97 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EXP-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Phase 3 - DistilBERT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DistilBERT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MRPC</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>3668</v>
+      </c>
+      <c r="G8" t="n">
+        <v>408</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1725</v>
+      </c>
+      <c r="I8" t="n">
+        <v>16</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2e-05</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.7971014492753623</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.8626023657870792</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.8265039232781168</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.8441674087266251</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.8784703891300609</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>209.4907968044281</v>
+      </c>
+      <c r="U8" t="n">
+        <v>4.201127290725708</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>DistilBERT fine-tuned on MRPC</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>